<commit_message>
Update completed budget review workbook export
</commit_message>
<xml_diff>
--- a/completed_budget_review.xlsx
+++ b/completed_budget_review.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Read Me" sheetId="1" r:id="Rbfd72184a55040da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Prior Year P&amp;L" sheetId="2" r:id="R0e42b8460dcb46e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Prior Year Sales" sheetId="3" r:id="R23527e2a431149ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Prior Year Marketing" sheetId="4" r:id="R543b03124b90425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prior Year Programs" sheetId="5" r:id="Rb2d6e46daea04bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Draft Sales Budget" sheetId="6" r:id="Rc573bcdc66504c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Draft Program Plan" sheetId="7" r:id="Ra2fc92eff9ab4715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Draft Operating Costs" sheetId="8" r:id="R4ca75fcb484b40d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Draft P&amp;L" sheetId="9" r:id="Rf8d1c8cc30944515"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Assumption Review" sheetId="11" r:id="Re28890f27a4948da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Corrected Budget" sheetId="12" r:id="Ra60610d0f6c040ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Management Recommendation" sheetId="13" r:id="Ra952f2ef1d314405"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Management Budget" sheetId="14" r:id="R62925ec26dea477e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Monthly Comparison" sheetId="15" r:id="R416b008aba614c07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Read Me" sheetId="1" r:id="R675a2e2e0b724f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Prior Year P&amp;L" sheetId="2" r:id="R5faea504d81a4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Prior Year Sales" sheetId="3" r:id="R7d6eb92943234f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Prior Year Marketing" sheetId="4" r:id="R913717175779466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prior Year Programs" sheetId="5" r:id="Rc0d1b6392aa44c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Draft Sales Budget" sheetId="6" r:id="R795ef286ab6d4d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Draft Program Plan" sheetId="7" r:id="R55b7e4a7562642c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Draft Operating Costs" sheetId="8" r:id="Ra496d3f4d1394f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Draft P&amp;L" sheetId="9" r:id="R5fb2e2e9d2f94845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Assumption Review" sheetId="11" r:id="R9465b3bb73b94dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Corrected Budget" sheetId="12" r:id="R5d8d43c22d77456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Management Recommendation" sheetId="13" r:id="Rd3738a983acf4c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Management Budget" sheetId="14" r:id="R9ebf005396ab42a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Monthly Comparison" sheetId="15" r:id="Ra399fcb89f3f46d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2056,9 +2056,7 @@
       <x:c r="I24" s="93" t="str"/>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="92" t="n">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="B25" s="92"/>
       <x:c r="C25" s="93" t="str"/>
       <x:c r="D25" s="93" t="str"/>
       <x:c r="E25" s="93" t="str"/>
@@ -2068,9 +2066,7 @@
       <x:c r="I25" s="93" t="str"/>
     </x:row>
     <x:row r="26">
-      <x:c r="B26" s="92" t="n">
-        <x:v>20</x:v>
-      </x:c>
+      <x:c r="B26" s="92"/>
       <x:c r="C26" s="93" t="str"/>
       <x:c r="D26" s="93" t="str"/>
       <x:c r="E26" s="93" t="str"/>
@@ -2216,39 +2212,51 @@
       </x:c>
       <x:c r="C5" s="194"/>
       <x:c r="D5" s="195" t="n">
+        <x:f>C28</x:f>
         <x:v>8600</x:v>
       </x:c>
       <x:c r="E5" s="195" t="n">
+        <x:f>D28</x:f>
         <x:v>12700</x:v>
       </x:c>
       <x:c r="F5" s="195" t="n">
+        <x:f>E28</x:f>
         <x:v>15000</x:v>
       </x:c>
       <x:c r="G5" s="195" t="n">
+        <x:f>F28</x:f>
         <x:v>12050</x:v>
       </x:c>
       <x:c r="H5" s="195" t="n">
+        <x:f>G28</x:f>
         <x:v>13300</x:v>
       </x:c>
       <x:c r="I5" s="195" t="n">
+        <x:f>H28</x:f>
         <x:v>12750</x:v>
       </x:c>
       <x:c r="J5" s="195" t="n">
+        <x:f>I28</x:f>
         <x:v>2500</x:v>
       </x:c>
       <x:c r="K5" s="195" t="n">
+        <x:f>J28</x:f>
         <x:v>9000</x:v>
       </x:c>
       <x:c r="L5" s="195" t="n">
+        <x:f>K28</x:f>
         <x:v>17000</x:v>
       </x:c>
       <x:c r="M5" s="195" t="n">
+        <x:f>L28</x:f>
         <x:v>19450</x:v>
       </x:c>
       <x:c r="N5" s="195" t="n">
+        <x:f>M28</x:f>
         <x:v>16800</x:v>
       </x:c>
       <x:c r="O5" s="195" t="n">
+        <x:f>N28</x:f>
         <x:v>7500</x:v>
       </x:c>
       <x:c r="P5" s="195" t="n">
@@ -2265,39 +2273,51 @@
         <x:v>Evidence / calculation</x:v>
       </x:c>
       <x:c r="D6" s="170" t="n">
+        <x:f>C29</x:f>
         <x:v>-4000</x:v>
       </x:c>
       <x:c r="E6" s="170" t="n">
+        <x:f>D29</x:f>
         <x:v>-5955</x:v>
       </x:c>
       <x:c r="F6" s="170" t="n">
+        <x:f>E29</x:f>
         <x:v>-6250</x:v>
       </x:c>
       <x:c r="G6" s="170" t="n">
+        <x:f>F29</x:f>
         <x:v>-6152.5</x:v>
       </x:c>
       <x:c r="H6" s="170" t="n">
+        <x:f>G29</x:f>
         <x:v>-4805</x:v>
       </x:c>
       <x:c r="I6" s="170" t="n">
+        <x:f>H29</x:f>
         <x:v>-8025</x:v>
       </x:c>
       <x:c r="J6" s="170" t="n">
+        <x:f>I29</x:f>
         <x:v>-1195</x:v>
       </x:c>
       <x:c r="K6" s="170" t="n">
+        <x:f>J29</x:f>
         <x:v>-4760</x:v>
       </x:c>
       <x:c r="L6" s="170" t="n">
+        <x:f>K29</x:f>
         <x:v>-6735</x:v>
       </x:c>
       <x:c r="M6" s="170" t="n">
+        <x:f>L29</x:f>
         <x:v>-8865</x:v>
       </x:c>
       <x:c r="N6" s="170" t="n">
+        <x:f>M29</x:f>
         <x:v>-8090</x:v>
       </x:c>
       <x:c r="O6" s="170" t="n">
+        <x:f>N29</x:f>
         <x:v>-4035</x:v>
       </x:c>
       <x:c r="P6" s="170" t="n">
@@ -2430,39 +2450,51 @@
       </x:c>
       <x:c r="C9" s="93" t="str"/>
       <x:c r="D9" s="190" t="n">
+        <x:f>C30</x:f>
         <x:v>-24725</x:v>
       </x:c>
       <x:c r="E9" s="190" t="n">
+        <x:f>D30</x:f>
         <x:v>-24225</x:v>
       </x:c>
       <x:c r="F9" s="190" t="n">
+        <x:f>E30</x:f>
         <x:v>-21975</x:v>
       </x:c>
       <x:c r="G9" s="190" t="n">
+        <x:f>F30</x:f>
         <x:v>-23275</x:v>
       </x:c>
       <x:c r="H9" s="190" t="n">
+        <x:f>G30</x:f>
         <x:v>-23641.67</x:v>
       </x:c>
       <x:c r="I9" s="190" t="n">
+        <x:f>H30</x:f>
         <x:v>-23141.67</x:v>
       </x:c>
       <x:c r="J9" s="190" t="n">
+        <x:f>I30</x:f>
         <x:v>-21641.67</x:v>
       </x:c>
       <x:c r="K9" s="190" t="n">
+        <x:f>J30</x:f>
         <x:v>-22641.67</x:v>
       </x:c>
       <x:c r="L9" s="190" t="n">
+        <x:f>K30</x:f>
         <x:v>-25141.67</x:v>
       </x:c>
       <x:c r="M9" s="190" t="n">
+        <x:f>L30</x:f>
         <x:v>-25641.67</x:v>
       </x:c>
       <x:c r="N9" s="190" t="n">
+        <x:f>M30</x:f>
         <x:v>-24641.67</x:v>
       </x:c>
       <x:c r="O9" s="190" t="n">
+        <x:f>N30</x:f>
         <x:v>-23141.67</x:v>
       </x:c>
       <x:c r="P9" s="190" t="n">
@@ -2595,56 +2627,56 @@
       </x:c>
       <x:c r="C12" s="93" t="str"/>
       <x:c r="D12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,D$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,E$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,F$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>4</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,G$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,H$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,I$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>4</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,J$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>1</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,J$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,K$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,L$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>6</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,M$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>5</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,N$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>5</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,O$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P12" s="190" t="n">
         <x:f>SUM(D12:O12)</x:f>
-        <x:v>43</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2654,56 +2686,56 @@
       </x:c>
       <x:c r="C13" s="93" t="str"/>
       <x:c r="D13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,D$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>18</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,E$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,F$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,G$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,H$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>18</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,I$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,J$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,J$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,K$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,L$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,M$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,N$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,O$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P13" s="190" t="n">
         <x:f>SUM(D13:O13)</x:f>
-        <x:v>136</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -3194,6 +3226,138 @@
       </x:c>
       <x:c r="N27" s="169" t="n">
         <x:v>-416.67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="166" t="str">
+        <x:v>Part 1 revenue used by P&amp;L</x:v>
+      </x:c>
+      <x:c r="B28" s="166" t="str">
+        <x:v>Supporting calculation: corrected register bridge</x:v>
+      </x:c>
+      <x:c r="C28" s="169" t="n">
+        <x:v>8600</x:v>
+      </x:c>
+      <x:c r="D28" s="169" t="n">
+        <x:v>12700</x:v>
+      </x:c>
+      <x:c r="E28" s="169" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="F28" s="169" t="n">
+        <x:v>12050</x:v>
+      </x:c>
+      <x:c r="G28" s="169" t="n">
+        <x:v>13300</x:v>
+      </x:c>
+      <x:c r="H28" s="169" t="n">
+        <x:v>12750</x:v>
+      </x:c>
+      <x:c r="I28" s="169" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="J28" s="169" t="n">
+        <x:v>9000</x:v>
+      </x:c>
+      <x:c r="K28" s="169" t="n">
+        <x:v>17000</x:v>
+      </x:c>
+      <x:c r="L28" s="169" t="n">
+        <x:v>19450</x:v>
+      </x:c>
+      <x:c r="M28" s="169" t="n">
+        <x:v>16800</x:v>
+      </x:c>
+      <x:c r="N28" s="169" t="n">
+        <x:v>7500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="166" t="str">
+        <x:v>Part 1 direct costs used by P&amp;L</x:v>
+      </x:c>
+      <x:c r="B29" s="166" t="str">
+        <x:v>Supporting calculation: corrected register cost bridge</x:v>
+      </x:c>
+      <x:c r="C29" s="169" t="n">
+        <x:v>-4000</x:v>
+      </x:c>
+      <x:c r="D29" s="169" t="n">
+        <x:v>-5955</x:v>
+      </x:c>
+      <x:c r="E29" s="169" t="n">
+        <x:v>-6250</x:v>
+      </x:c>
+      <x:c r="F29" s="169" t="n">
+        <x:v>-6152.5</x:v>
+      </x:c>
+      <x:c r="G29" s="169" t="n">
+        <x:v>-4805</x:v>
+      </x:c>
+      <x:c r="H29" s="169" t="n">
+        <x:v>-8025</x:v>
+      </x:c>
+      <x:c r="I29" s="169" t="n">
+        <x:v>-1195</x:v>
+      </x:c>
+      <x:c r="J29" s="169" t="n">
+        <x:v>-4760</x:v>
+      </x:c>
+      <x:c r="K29" s="169" t="n">
+        <x:v>-6735</x:v>
+      </x:c>
+      <x:c r="L29" s="169" t="n">
+        <x:v>-8865</x:v>
+      </x:c>
+      <x:c r="M29" s="169" t="n">
+        <x:v>-8090</x:v>
+      </x:c>
+      <x:c r="N29" s="169" t="n">
+        <x:v>-4035</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="166" t="str">
+        <x:v>Part 1 operating costs used by P&amp;L</x:v>
+      </x:c>
+      <x:c r="B30" s="166" t="str">
+        <x:v>Supporting calculation: operating-cost bridge and timing corrections</x:v>
+      </x:c>
+      <x:c r="C30" s="169" t="n">
+        <x:v>-24725</x:v>
+      </x:c>
+      <x:c r="D30" s="169" t="n">
+        <x:v>-24225</x:v>
+      </x:c>
+      <x:c r="E30" s="169" t="n">
+        <x:v>-21975</x:v>
+      </x:c>
+      <x:c r="F30" s="169" t="n">
+        <x:v>-23275</x:v>
+      </x:c>
+      <x:c r="G30" s="169" t="n">
+        <x:v>-23641.67</x:v>
+      </x:c>
+      <x:c r="H30" s="169" t="n">
+        <x:v>-23141.67</x:v>
+      </x:c>
+      <x:c r="I30" s="169" t="n">
+        <x:v>-21641.67</x:v>
+      </x:c>
+      <x:c r="J30" s="169" t="n">
+        <x:v>-22641.67</x:v>
+      </x:c>
+      <x:c r="K30" s="169" t="n">
+        <x:v>-25141.67</x:v>
+      </x:c>
+      <x:c r="L30" s="169" t="n">
+        <x:v>-25641.67</x:v>
+      </x:c>
+      <x:c r="M30" s="169" t="n">
+        <x:v>-24641.67</x:v>
+      </x:c>
+      <x:c r="N30" s="169" t="n">
+        <x:v>-23141.67</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3679,39 +3843,51 @@
       </x:c>
       <x:c r="C5" s="194"/>
       <x:c r="D5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!D5+C17</x:f>
         <x:v>8600</x:v>
       </x:c>
       <x:c r="E5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!E5+D17</x:f>
         <x:v>12700</x:v>
       </x:c>
       <x:c r="F5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!F5+E17</x:f>
         <x:v>15000</x:v>
       </x:c>
       <x:c r="G5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!G5+F17</x:f>
         <x:v>12050</x:v>
       </x:c>
       <x:c r="H5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!H5+G17</x:f>
         <x:v>13300</x:v>
       </x:c>
       <x:c r="I5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!I5+H17</x:f>
         <x:v>22750</x:v>
       </x:c>
       <x:c r="J5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!J5+I17</x:f>
         <x:v>12500</x:v>
       </x:c>
       <x:c r="K5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!K5+J17</x:f>
         <x:v>19000</x:v>
       </x:c>
       <x:c r="L5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!L5+K17</x:f>
         <x:v>27000</x:v>
       </x:c>
       <x:c r="M5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!M5+L17</x:f>
         <x:v>29450</x:v>
       </x:c>
       <x:c r="N5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!N5+M17</x:f>
         <x:v>26800</x:v>
       </x:c>
       <x:c r="O5" s="195" t="n">
+        <x:f>'10 Corrected Budget'!O5+N17</x:f>
         <x:v>17500</x:v>
       </x:c>
       <x:c r="P5" s="195" t="n">
@@ -3728,39 +3904,51 @@
         <x:v>Decision / calculation</x:v>
       </x:c>
       <x:c r="D6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!D6+C18+C19</x:f>
         <x:v>-1900</x:v>
       </x:c>
       <x:c r="E6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!E6+D18+D19</x:f>
         <x:v>-3855</x:v>
       </x:c>
       <x:c r="F6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!F6+E18+E19</x:f>
         <x:v>-3450</x:v>
       </x:c>
       <x:c r="G6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!G6+F18+F19</x:f>
         <x:v>-4053</x:v>
       </x:c>
       <x:c r="H6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!H6+G18+G19</x:f>
         <x:v>-2705</x:v>
       </x:c>
       <x:c r="I6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!I6+H18+H19</x:f>
         <x:v>-6225</x:v>
       </x:c>
       <x:c r="J6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!J6+I18+I19</x:f>
         <x:v>-1425</x:v>
       </x:c>
       <x:c r="K6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!K6+J18+J19</x:f>
         <x:v>-3450</x:v>
       </x:c>
       <x:c r="L6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!L6+K18+K19</x:f>
         <x:v>-4655</x:v>
       </x:c>
       <x:c r="M6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!M6+L18+L19</x:f>
         <x:v>-6015</x:v>
       </x:c>
       <x:c r="N6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!N6+M18+M19</x:f>
         <x:v>-6780</x:v>
       </x:c>
       <x:c r="O6" s="243" t="n">
+        <x:f>'10 Corrected Budget'!O6+N18+N19</x:f>
         <x:v>-2725</x:v>
       </x:c>
       <x:c r="P6" s="243" t="n">
@@ -4070,56 +4258,56 @@
       </x:c>
       <x:c r="C12" s="93"/>
       <x:c r="D12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,D$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,E$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,F$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>4</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,G$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,H$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,I$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>4</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,J$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>1</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,J$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,K$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,L$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>6</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,M$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>5</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,N$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>5</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O12" s="190" t="n">
-        <x:f>SUMIF('06 Draft Program Plan'!$C$7:$C$32,O$4,'06 Draft Program Plan'!$G$7:$G$32)</x:f>
-        <x:v>3</x:v>
+        <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P12" s="190" t="n">
         <x:f>SUM(D12:O12)</x:f>
-        <x:v>43</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4129,56 +4317,56 @@
       </x:c>
       <x:c r="C13" s="93"/>
       <x:c r="D13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,D$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>18</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,E$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,F$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,G$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,H$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>18</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,I$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,J$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,J$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,K$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,L$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,M$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,N$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
-        <x:v>20</x:v>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="O13" s="190" t="n">
-        <x:f>SUMIFS('06 Draft Program Plan'!$H$7:$H$32,'06 Draft Program Plan'!$C$7:$C$32,O$4,'06 Draft Program Plan'!$F$7:$F$32,"Open")</x:f>
+        <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P13" s="190" t="n">
         <x:f>SUM(D13:O13)</x:f>
-        <x:v>136</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>

<commit_message>
Add recalculation metadata and capacity caches to Excel export
</commit_message>
<xml_diff>
--- a/completed_budget_review.xlsx
+++ b/completed_budget_review.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Read Me" sheetId="1" r:id="R675a2e2e0b724f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Prior Year P&amp;L" sheetId="2" r:id="R5faea504d81a4b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Prior Year Sales" sheetId="3" r:id="R7d6eb92943234f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Prior Year Marketing" sheetId="4" r:id="R913717175779466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prior Year Programs" sheetId="5" r:id="Rc0d1b6392aa44c10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Draft Sales Budget" sheetId="6" r:id="R795ef286ab6d4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Draft Program Plan" sheetId="7" r:id="R55b7e4a7562642c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Draft Operating Costs" sheetId="8" r:id="Ra496d3f4d1394f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Draft P&amp;L" sheetId="9" r:id="R5fb2e2e9d2f94845"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Assumption Review" sheetId="11" r:id="R9465b3bb73b94dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Corrected Budget" sheetId="12" r:id="R5d8d43c22d77456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Management Recommendation" sheetId="13" r:id="Rd3738a983acf4c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Management Budget" sheetId="14" r:id="R9ebf005396ab42a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Monthly Comparison" sheetId="15" r:id="Ra399fcb89f3f46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Read Me" sheetId="1" r:id="R4bc0c4b180ed4932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Prior Year P&amp;L" sheetId="2" r:id="R230dbe7e52a04458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Prior Year Sales" sheetId="3" r:id="R72cf711b92df4a55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Prior Year Marketing" sheetId="4" r:id="R4fdbfabbf1394a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prior Year Programs" sheetId="5" r:id="R5cab524fb4af4ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Draft Sales Budget" sheetId="6" r:id="Rfd44844c84e7427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Draft Program Plan" sheetId="7" r:id="R54d14459818e40a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Draft Operating Costs" sheetId="8" r:id="R9fa34d5f6f7741ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Draft P&amp;L" sheetId="9" r:id="R38de045575bf42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Assumption Review" sheetId="11" r:id="R37c732d149cf457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Corrected Budget" sheetId="12" r:id="R133c30bdacf14646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Management Recommendation" sheetId="13" r:id="R8470bc85bc2c43cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Management Budget" sheetId="14" r:id="R853715b850714497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Monthly Comparison" sheetId="15" r:id="Rd2d14043d6d6425f"/>
   </x:sheets>
+  <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </x:workbook>
 </file>
 
@@ -2628,55 +2629,55 @@
       <x:c r="C12" s="93" t="str"/>
       <x:c r="D12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,J$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P12" s="190" t="n">
         <x:f>SUM(D12:O12)</x:f>
-        <x:v>0</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2687,7 +2688,7 @@
       <x:c r="C13" s="93" t="str"/>
       <x:c r="D13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -2695,7 +2696,7 @@
       </x:c>
       <x:c r="F13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -2703,7 +2704,7 @@
       </x:c>
       <x:c r="H13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="I13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -2715,19 +2716,19 @@
       </x:c>
       <x:c r="K13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="M13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="N13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="O13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -2735,7 +2736,7 @@
       </x:c>
       <x:c r="P13" s="190" t="n">
         <x:f>SUM(D13:O13)</x:f>
-        <x:v>0</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4259,55 +4260,55 @@
       <x:c r="C12" s="93"/>
       <x:c r="D12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,J$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="L12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O12" s="190" t="n">
         <x:f>SUMIF('06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$F$7:$F$32)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="P12" s="190" t="n">
         <x:f>SUM(D12:O12)</x:f>
-        <x:v>0</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4318,7 +4319,7 @@
       <x:c r="C13" s="93"/>
       <x:c r="D13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,D$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,E$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -4326,7 +4327,7 @@
       </x:c>
       <x:c r="F13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,F$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,G$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -4334,7 +4335,7 @@
       </x:c>
       <x:c r="H13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,H$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="I13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,I$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -4346,19 +4347,19 @@
       </x:c>
       <x:c r="K13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,K$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,L$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="M13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,M$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="N13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,N$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="O13" s="190" t="n">
         <x:f>SUMIFS('06 Draft Program Plan'!$G$7:$G$32,'06 Draft Program Plan'!$B$7:$B$32,O$4,'06 Draft Program Plan'!$E$7:$E$32,"Open")</x:f>
@@ -4366,7 +4367,7 @@
       </x:c>
       <x:c r="P13" s="190" t="n">
         <x:f>SUM(D13:O13)</x:f>
-        <x:v>0</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>